<commit_message>
- fixed typo maxiumum in LG file size error message (#350)
</commit_message>
<xml_diff>
--- a/source/Translation (IT).xlsx
+++ b/source/Translation (IT).xlsx
@@ -5477,7 +5477,7 @@
     <t xml:space="preserve">TllFileSerializerPlugin_ERR_fileTooBig</t>
   </si>
   <si>
-    <t xml:space="preserve">File size {0} is larger than allowed maxiumum of {1}</t>
+    <t xml:space="preserve">File size {0} is larger than allowed maximum of {1}</t>
   </si>
   <si>
     <t xml:space="preserve">La dimensione del file {0} è maggiore del massimo consentito di {1}</t>
@@ -5489,7 +5489,7 @@
     <t xml:space="preserve">Dateigröße {0} überschreitet das erlaubte Maximum von {1}</t>
   </si>
   <si>
-    <t xml:space="preserve">Dimensiunea fișierului {0} este mai mare decât permisiunea maxiumum din {1}</t>
+    <t xml:space="preserve">Dimensiunea fișierului {0} este mai mare decât permisiunea maximum din {1}</t>
   </si>
   <si>
     <t xml:space="preserve">TllFileSerializer_ERR_dupeChannel</t>

</xml_diff>